<commit_message>
update Wed 03 25
</commit_message>
<xml_diff>
--- a/files/sql/update trx_group_user.xlsx
+++ b/files/sql/update trx_group_user.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rafli\OneDrive\Desktop\aaa\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Danu\repo\golang\promise-migration\files\sql\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CB43FCF-A02B-4126-A79A-964AD9CAF470}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE648A48-F41A-4A64-AF5C-7F00CB5AA2DB}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="132" yWindow="0" windowWidth="22908" windowHeight="12960" activeTab="2" xr2:uid="{59E1CA53-7D92-4E29-AF1C-85F41487F742}"/>
+    <workbookView xWindow="132" yWindow="0" windowWidth="22908" windowHeight="12960" xr2:uid="{59E1CA53-7D92-4E29-AF1C-85F41487F742}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="63">
   <si>
     <t>ihrom-lestari@ecampus.ut.ac.id</t>
   </si>
@@ -192,6 +192,36 @@
   </si>
   <si>
     <t>12345654321</t>
+  </si>
+  <si>
+    <t>nama</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>nip</t>
+  </si>
+  <si>
+    <t>kode_unit_pbj</t>
+  </si>
+  <si>
+    <t>kode_jabatan</t>
+  </si>
+  <si>
+    <t>status_aktif</t>
+  </si>
+  <si>
+    <t>sk</t>
+  </si>
+  <si>
+    <t>encrypt_key</t>
+  </si>
+  <si>
+    <t>kode_unit</t>
+  </si>
+  <si>
+    <t>nama_unit</t>
   </si>
 </sst>
 </file>
@@ -234,7 +264,77 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="24">
+  <dxfs count="31">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -785,7 +885,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E1FB5DF-4EF9-419C-B3F9-DDD094F1488E}">
-  <dimension ref="B3:H119"/>
+  <dimension ref="B3:H124"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="28.6640625" bestFit="1" customWidth="1"/>
@@ -2208,7 +2308,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="97" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B97" t="s">
         <v>19</v>
       </c>
@@ -2225,7 +2325,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="98" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B98" t="s">
         <v>19</v>
       </c>
@@ -2242,41 +2342,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="99" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B99" t="s">
-        <v>20</v>
-      </c>
-      <c r="C99">
-        <v>4883</v>
-      </c>
-      <c r="D99" t="s">
-        <v>6</v>
-      </c>
-      <c r="E99">
-        <v>32728</v>
-      </c>
-      <c r="F99">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="100" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B100" t="s">
-        <v>20</v>
-      </c>
-      <c r="C100">
-        <v>11550</v>
-      </c>
-      <c r="D100" t="s">
-        <v>7</v>
-      </c>
-      <c r="E100">
-        <v>32728</v>
-      </c>
-      <c r="F100">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="104" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="104" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B104" t="s">
         <v>17</v>
       </c>
@@ -2293,7 +2359,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="105" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B105" t="s">
         <v>17</v>
       </c>
@@ -2310,7 +2376,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="106" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B106" t="s">
         <v>18</v>
       </c>
@@ -2327,7 +2393,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="107" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="107" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B107" t="s">
         <v>18</v>
       </c>
@@ -2344,7 +2410,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="108" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B108" t="s">
         <v>19</v>
       </c>
@@ -2361,7 +2427,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="109" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="109" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B109" t="s">
         <v>19</v>
       </c>
@@ -2378,67 +2444,21 @@
         <v>1</v>
       </c>
     </row>
-    <row r="110" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B110" t="s">
-        <v>20</v>
-      </c>
-      <c r="C110">
-        <v>66810</v>
-      </c>
-      <c r="D110" t="s">
-        <v>13</v>
-      </c>
-      <c r="E110">
-        <v>32728</v>
-      </c>
-      <c r="F110">
-        <v>1</v>
-      </c>
-      <c r="H110" t="str">
-        <f t="shared" ref="H110:H119" si="9">"INSERT INTO trx_group_user (kode_group,id_user, status) VALUES ('"&amp;D110&amp;"', "&amp;E110&amp;", '"&amp;F110&amp;"');"</f>
-        <v>INSERT INTO trx_group_user (kode_group,id_user, status) VALUES ('G03.2     ', 32728, '1');</v>
-      </c>
-    </row>
-    <row r="111" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B111" t="s">
-        <v>20</v>
-      </c>
-      <c r="C111">
-        <v>66811</v>
-      </c>
-      <c r="D111" t="s">
-        <v>21</v>
-      </c>
-      <c r="E111">
-        <v>32728</v>
-      </c>
-      <c r="F111">
-        <v>1</v>
-      </c>
-      <c r="H111" t="str">
-        <f t="shared" si="9"/>
-        <v>INSERT INTO trx_group_user (kode_group,id_user, status) VALUES ('G00.6     ', 32728, '1');</v>
-      </c>
-    </row>
-    <row r="112" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="112" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B112" t="s">
         <v>20</v>
       </c>
       <c r="C112">
-        <v>66812</v>
+        <v>4883</v>
       </c>
       <c r="D112" t="s">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="E112">
         <v>32728</v>
       </c>
       <c r="F112">
         <v>1</v>
-      </c>
-      <c r="H112" t="str">
-        <f t="shared" si="9"/>
-        <v>INSERT INTO trx_group_user (kode_group,id_user, status) VALUES ('G11.2     ', 32728, '1');</v>
       </c>
     </row>
     <row r="113" spans="2:8" x14ac:dyDescent="0.3">
@@ -2446,7 +2466,7 @@
         <v>20</v>
       </c>
       <c r="C113">
-        <v>66813</v>
+        <v>11550</v>
       </c>
       <c r="D113" t="s">
         <v>7</v>
@@ -2456,27 +2476,6 @@
       </c>
       <c r="F113">
         <v>1</v>
-      </c>
-    </row>
-    <row r="114" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B114" t="s">
-        <v>20</v>
-      </c>
-      <c r="C114">
-        <v>66814</v>
-      </c>
-      <c r="D114" t="s">
-        <v>28</v>
-      </c>
-      <c r="E114">
-        <v>32728</v>
-      </c>
-      <c r="F114">
-        <v>1</v>
-      </c>
-      <c r="H114" t="str">
-        <f t="shared" si="9"/>
-        <v>INSERT INTO trx_group_user (kode_group,id_user, status) VALUES ('G11.4     ', 32728, '1');</v>
       </c>
     </row>
     <row r="115" spans="2:8" x14ac:dyDescent="0.3">
@@ -2484,10 +2483,10 @@
         <v>20</v>
       </c>
       <c r="C115">
-        <v>66815</v>
+        <v>66810</v>
       </c>
       <c r="D115" t="s">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="E115">
         <v>32728</v>
@@ -2496,8 +2495,8 @@
         <v>1</v>
       </c>
       <c r="H115" t="str">
-        <f t="shared" si="9"/>
-        <v>INSERT INTO trx_group_user (kode_group,id_user, status) VALUES ('G04.2     ', 32728, '1');</v>
+        <f t="shared" ref="H115:H124" si="9">"INSERT INTO trx_group_user (kode_group,id_user, status) VALUES ('"&amp;D115&amp;"', "&amp;E115&amp;", '"&amp;F115&amp;"');"</f>
+        <v>INSERT INTO trx_group_user (kode_group,id_user, status) VALUES ('G03.2     ', 32728, '1');</v>
       </c>
     </row>
     <row r="116" spans="2:8" x14ac:dyDescent="0.3">
@@ -2505,10 +2504,10 @@
         <v>20</v>
       </c>
       <c r="C116">
-        <v>66816</v>
+        <v>66811</v>
       </c>
       <c r="D116" t="s">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="E116">
         <v>32728</v>
@@ -2518,7 +2517,7 @@
       </c>
       <c r="H116" t="str">
         <f t="shared" si="9"/>
-        <v>INSERT INTO trx_group_user (kode_group,id_user, status) VALUES ('G01.4     ', 32728, '1');</v>
+        <v>INSERT INTO trx_group_user (kode_group,id_user, status) VALUES ('G00.6     ', 32728, '1');</v>
       </c>
     </row>
     <row r="117" spans="2:8" x14ac:dyDescent="0.3">
@@ -2526,10 +2525,10 @@
         <v>20</v>
       </c>
       <c r="C117">
-        <v>66817</v>
+        <v>66812</v>
       </c>
       <c r="D117" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="E117">
         <v>32728</v>
@@ -2539,7 +2538,7 @@
       </c>
       <c r="H117" t="str">
         <f t="shared" si="9"/>
-        <v>INSERT INTO trx_group_user (kode_group,id_user, status) VALUES ('G03.1     ', 32728, '1');</v>
+        <v>INSERT INTO trx_group_user (kode_group,id_user, status) VALUES ('G11.2     ', 32728, '1');</v>
       </c>
     </row>
     <row r="118" spans="2:8" x14ac:dyDescent="0.3">
@@ -2547,20 +2546,16 @@
         <v>20</v>
       </c>
       <c r="C118">
-        <v>66818</v>
+        <v>66813</v>
       </c>
       <c r="D118" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E118">
         <v>32728</v>
       </c>
       <c r="F118">
         <v>1</v>
-      </c>
-      <c r="H118" t="str">
-        <f t="shared" si="9"/>
-        <v>INSERT INTO trx_group_user (kode_group,id_user, status) VALUES ('G04.5     ', 32728, '1');</v>
       </c>
     </row>
     <row r="119" spans="2:8" x14ac:dyDescent="0.3">
@@ -2568,10 +2563,10 @@
         <v>20</v>
       </c>
       <c r="C119">
-        <v>66819</v>
+        <v>66814</v>
       </c>
       <c r="D119" t="s">
-        <v>2</v>
+        <v>28</v>
       </c>
       <c r="E119">
         <v>32728</v>
@@ -2581,27 +2576,138 @@
       </c>
       <c r="H119" t="str">
         <f t="shared" si="9"/>
+        <v>INSERT INTO trx_group_user (kode_group,id_user, status) VALUES ('G11.4     ', 32728, '1');</v>
+      </c>
+    </row>
+    <row r="120" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B120" t="s">
+        <v>20</v>
+      </c>
+      <c r="C120">
+        <v>66815</v>
+      </c>
+      <c r="D120" t="s">
+        <v>35</v>
+      </c>
+      <c r="E120">
+        <v>32728</v>
+      </c>
+      <c r="F120">
+        <v>1</v>
+      </c>
+      <c r="H120" t="str">
+        <f t="shared" si="9"/>
+        <v>INSERT INTO trx_group_user (kode_group,id_user, status) VALUES ('G04.2     ', 32728, '1');</v>
+      </c>
+    </row>
+    <row r="121" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B121" t="s">
+        <v>20</v>
+      </c>
+      <c r="C121">
+        <v>66816</v>
+      </c>
+      <c r="D121" t="s">
+        <v>4</v>
+      </c>
+      <c r="E121">
+        <v>32728</v>
+      </c>
+      <c r="F121">
+        <v>1</v>
+      </c>
+      <c r="H121" t="str">
+        <f t="shared" si="9"/>
+        <v>INSERT INTO trx_group_user (kode_group,id_user, status) VALUES ('G01.4     ', 32728, '1');</v>
+      </c>
+    </row>
+    <row r="122" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B122" t="s">
+        <v>20</v>
+      </c>
+      <c r="C122">
+        <v>66817</v>
+      </c>
+      <c r="D122" t="s">
+        <v>33</v>
+      </c>
+      <c r="E122">
+        <v>32728</v>
+      </c>
+      <c r="F122">
+        <v>1</v>
+      </c>
+      <c r="H122" t="str">
+        <f t="shared" si="9"/>
+        <v>INSERT INTO trx_group_user (kode_group,id_user, status) VALUES ('G03.1     ', 32728, '1');</v>
+      </c>
+    </row>
+    <row r="123" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B123" t="s">
+        <v>20</v>
+      </c>
+      <c r="C123">
+        <v>66818</v>
+      </c>
+      <c r="D123" t="s">
+        <v>3</v>
+      </c>
+      <c r="E123">
+        <v>32728</v>
+      </c>
+      <c r="F123">
+        <v>1</v>
+      </c>
+      <c r="H123" t="str">
+        <f t="shared" si="9"/>
+        <v>INSERT INTO trx_group_user (kode_group,id_user, status) VALUES ('G04.5     ', 32728, '1');</v>
+      </c>
+    </row>
+    <row r="124" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B124" t="s">
+        <v>20</v>
+      </c>
+      <c r="C124">
+        <v>66819</v>
+      </c>
+      <c r="D124" t="s">
+        <v>2</v>
+      </c>
+      <c r="E124">
+        <v>32728</v>
+      </c>
+      <c r="F124">
+        <v>1</v>
+      </c>
+      <c r="H124" t="str">
+        <f t="shared" si="9"/>
         <v>INSERT INTO trx_group_user (kode_group,id_user, status) VALUES ('G05.5     ', 32728, '1');</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="D3:D30">
-    <cfRule type="duplicateValues" dxfId="9" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D32:D37">
-    <cfRule type="duplicateValues" dxfId="8" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D39:D58">
-    <cfRule type="duplicateValues" dxfId="7" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D60:D77">
-    <cfRule type="duplicateValues" dxfId="6" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D80:D84">
-    <cfRule type="duplicateValues" dxfId="5" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="4"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D93:D119">
-    <cfRule type="duplicateValues" dxfId="4" priority="1"/>
+  <conditionalFormatting sqref="D93:D98 D101:D111">
+    <cfRule type="duplicateValues" dxfId="9" priority="3"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D128:D138">
+    <cfRule type="duplicateValues" dxfId="8" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D112:D124">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3439,10 +3545,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="G9:G20">
-    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="G22:G29">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="29" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -3451,250 +3557,258 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47115FCB-453E-41C7-81F4-B34B28F24DFE}">
-  <dimension ref="B2:L9"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="2" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B2">
-        <v>2634</v>
-      </c>
-      <c r="C2" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F1" t="s">
+        <v>58</v>
+      </c>
+      <c r="G1" t="s">
+        <v>59</v>
+      </c>
+      <c r="H1" t="s">
+        <v>60</v>
+      </c>
+      <c r="I1" t="s">
+        <v>61</v>
+      </c>
+      <c r="J1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>46</v>
       </c>
-      <c r="D2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E2" s="1" t="s">
+      <c r="B2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-      <c r="G2">
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
         <v>39</v>
       </c>
-      <c r="H2" t="b">
-        <v>1</v>
-      </c>
-      <c r="K2" t="s">
+      <c r="F2" t="b">
+        <v>1</v>
+      </c>
+      <c r="I2" t="s">
         <v>37</v>
       </c>
-      <c r="L2" t="s">
+      <c r="J2" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B3">
-        <v>2635</v>
-      </c>
-      <c r="C3" t="s">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>46</v>
       </c>
-      <c r="D3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E3" s="1" t="s">
+      <c r="B3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
-      <c r="G3">
-        <v>1</v>
-      </c>
-      <c r="H3" t="b">
-        <v>1</v>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" t="s">
+        <v>47</v>
+      </c>
+      <c r="H3" t="s">
+        <v>48</v>
       </c>
       <c r="I3" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="J3" t="s">
-        <v>48</v>
-      </c>
-      <c r="K3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>4</v>
+      </c>
+      <c r="F4" t="b">
+        <v>1</v>
+      </c>
+      <c r="I4" t="s">
         <v>37</v>
       </c>
-      <c r="L3" t="s">
+      <c r="J4" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B4">
-        <v>2643</v>
-      </c>
-      <c r="C4" t="s">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>51</v>
       </c>
-      <c r="D4" t="s">
+      <c r="B5" t="s">
         <v>20</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="C5" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="F4">
-        <v>1</v>
-      </c>
-      <c r="G4">
-        <v>4</v>
-      </c>
-      <c r="H4" t="b">
-        <v>1</v>
-      </c>
-      <c r="K4" t="s">
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>7</v>
+      </c>
+      <c r="F5" t="b">
+        <v>1</v>
+      </c>
+      <c r="I5" t="s">
         <v>37</v>
       </c>
-      <c r="L4" t="s">
+      <c r="J5" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B5">
-        <v>2639</v>
-      </c>
-      <c r="C5" t="s">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>51</v>
       </c>
-      <c r="D5" t="s">
+      <c r="B6" t="s">
         <v>20</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="C6" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="F5">
-        <v>1</v>
-      </c>
-      <c r="G5">
-        <v>7</v>
-      </c>
-      <c r="H5" t="b">
-        <v>1</v>
-      </c>
-      <c r="K5" t="s">
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>6</v>
+      </c>
+      <c r="F6" t="b">
+        <v>1</v>
+      </c>
+      <c r="I6" t="s">
         <v>37</v>
       </c>
-      <c r="L5" t="s">
+      <c r="J6" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B6">
-        <v>2640</v>
-      </c>
-      <c r="C6" t="s">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>51</v>
       </c>
-      <c r="D6" t="s">
+      <c r="B7" t="s">
         <v>20</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="C7" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="F6">
-        <v>1</v>
-      </c>
-      <c r="G6">
-        <v>6</v>
-      </c>
-      <c r="H6" t="b">
-        <v>1</v>
-      </c>
-      <c r="K6" t="s">
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>35</v>
+      </c>
+      <c r="F7" t="b">
+        <v>1</v>
+      </c>
+      <c r="I7" t="s">
         <v>37</v>
       </c>
-      <c r="L6" t="s">
+      <c r="J7" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B7">
-        <v>2641</v>
-      </c>
-      <c r="C7" t="s">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
         <v>51</v>
       </c>
-      <c r="D7" t="s">
+      <c r="B8" t="s">
         <v>20</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="C8" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="F7">
-        <v>1</v>
-      </c>
-      <c r="G7">
-        <v>35</v>
-      </c>
-      <c r="H7" t="b">
-        <v>1</v>
-      </c>
-      <c r="K7" t="s">
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>8</v>
+      </c>
+      <c r="F8" t="b">
+        <v>1</v>
+      </c>
+      <c r="I8" t="s">
         <v>37</v>
       </c>
-      <c r="L7" t="s">
+      <c r="J8" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B8">
-        <v>2642</v>
-      </c>
-      <c r="C8" t="s">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>51</v>
       </c>
-      <c r="D8" t="s">
+      <c r="B9" t="s">
         <v>20</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="F8">
-        <v>1</v>
-      </c>
-      <c r="G8">
-        <v>8</v>
-      </c>
-      <c r="H8" t="b">
-        <v>1</v>
-      </c>
-      <c r="K8" t="s">
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9" t="b">
+        <v>1</v>
+      </c>
+      <c r="I9" t="s">
         <v>37</v>
       </c>
-      <c r="L8" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B9">
-        <v>2638</v>
-      </c>
-      <c r="C9" t="s">
-        <v>51</v>
-      </c>
-      <c r="D9" t="s">
-        <v>20</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F9">
-        <v>1</v>
-      </c>
-      <c r="G9">
-        <v>1</v>
-      </c>
-      <c r="H9" t="b">
-        <v>1</v>
-      </c>
-      <c r="K9" t="s">
+      <c r="J9" t="s">
         <v>37</v>
       </c>
-      <c r="L9" t="s">
-        <v>37</v>
-      </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="G2:G3">
-    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
+  <conditionalFormatting sqref="E2:E3">
+    <cfRule type="duplicateValues" dxfId="28" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>